<commit_message>
fixed paired plots for temp behavior
</commit_message>
<xml_diff>
--- a/data/temp_behavior.xlsx
+++ b/data/temp_behavior.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickhousley/GaTech Dropbox/CoS/BioSci/BioSci-Housley_Lab/04-papers/acute_ox/acute_oxaliplatin_encoding/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE16507-7D83-0A4B-A59D-AC158E574338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA555DE7-14A8-9D46-B467-0E62784EF2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15840" xr2:uid="{409C6191-3028-4579-A749-687FFA0974B0}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{409C6191-3028-4579-A749-687FFA0974B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="91">
   <si>
     <t>temp</t>
   </si>
@@ -107,9 +107,6 @@
     <t>ox 0 9-14</t>
   </si>
   <si>
-    <t>control 25 9-12 no mark</t>
-  </si>
-  <si>
     <t>control 0 9-13 no mark</t>
   </si>
   <si>
@@ -252,6 +249,66 @@
   </si>
   <si>
     <t>file_name_date</t>
+  </si>
+  <si>
+    <t>control 25 9-18</t>
+  </si>
+  <si>
+    <t>control 25 9-13 no mark</t>
+  </si>
+  <si>
+    <t>A100495-23-94</t>
+  </si>
+  <si>
+    <t>A100495-23-93</t>
+  </si>
+  <si>
+    <t>A100495-23-92</t>
+  </si>
+  <si>
+    <t>A100495-23-91</t>
+  </si>
+  <si>
+    <t>A100495-23-90</t>
+  </si>
+  <si>
+    <t>A100495-23-89</t>
+  </si>
+  <si>
+    <t>A100495-23-88</t>
+  </si>
+  <si>
+    <t>A100495-23-85</t>
+  </si>
+  <si>
+    <t>A100495-23-84</t>
+  </si>
+  <si>
+    <t>A100495-23-83</t>
+  </si>
+  <si>
+    <t>A100495-23-80</t>
+  </si>
+  <si>
+    <t>A100495-23-78</t>
+  </si>
+  <si>
+    <t>A100495-23-77</t>
+  </si>
+  <si>
+    <t>A100495-23-74</t>
+  </si>
+  <si>
+    <t>A100495-23-73</t>
+  </si>
+  <si>
+    <t>A100495-23-72</t>
+  </si>
+  <si>
+    <t>A100495-23-71</t>
+  </si>
+  <si>
+    <t>animalID</t>
   </si>
 </sst>
 </file>
@@ -612,32 +669,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFDEA3FA-602C-4935-8B74-4DEDB7BDAEDB}">
-  <dimension ref="A1:F418"/>
+  <dimension ref="A1:G418"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.33203125" customWidth="1"/>
     <col min="3" max="3" width="27.5" customWidth="1"/>
-    <col min="5" max="7" width="11.1640625" customWidth="1"/>
+    <col min="5" max="6" width="11.1640625" customWidth="1"/>
+    <col min="7" max="7" width="20.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>68</v>
       </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>69</v>
       </c>
-      <c r="F1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -656,8 +717,11 @@
       <c r="F2">
         <v>60</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -676,8 +740,11 @@
       <c r="F3">
         <v>25.63</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -696,8 +763,11 @@
       <c r="F4">
         <v>48.92</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -716,8 +786,11 @@
       <c r="F5">
         <v>27.63</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -736,8 +809,11 @@
       <c r="F6">
         <v>37.15</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -756,8 +832,11 @@
       <c r="F7">
         <v>37.799999999999997</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -776,8 +855,11 @@
       <c r="F8">
         <v>31.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -796,8 +878,11 @@
       <c r="F9">
         <v>35.78</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -816,8 +901,11 @@
       <c r="F10">
         <v>58.29</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -836,8 +924,11 @@
       <c r="F11">
         <v>47.980000000000004</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -856,8 +947,11 @@
       <c r="F12">
         <v>51.12</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -876,8 +970,11 @@
       <c r="F13">
         <v>37.049999999999997</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -896,8 +993,11 @@
       <c r="F14">
         <v>33.220000000000006</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -916,8 +1016,11 @@
       <c r="F15">
         <v>20.520000000000003</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -925,7 +1028,7 @@
         <v>797</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="D16">
         <v>25</v>
@@ -936,8 +1039,11 @@
       <c r="F16">
         <v>54.28</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -945,7 +1051,7 @@
         <v>6340</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -956,8 +1062,11 @@
       <c r="F17">
         <v>14.190000000000001</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -976,8 +1085,11 @@
       <c r="F18">
         <v>52.34</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -996,8 +1108,11 @@
       <c r="F19">
         <v>22.39</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1016,8 +1131,11 @@
       <c r="F20">
         <v>18.059999999999999</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1036,8 +1154,11 @@
       <c r="F21">
         <v>27.01</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1056,8 +1177,11 @@
       <c r="F22">
         <v>40.21</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1076,8 +1200,11 @@
       <c r="F23">
         <v>37.15</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G23" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1085,7 +1212,7 @@
         <v>9771</v>
       </c>
       <c r="C24" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="D24">
         <v>25</v>
@@ -1096,8 +1223,11 @@
       <c r="F24">
         <v>38.79</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G24" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1105,7 +1235,7 @@
         <v>4009</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -1116,8 +1246,11 @@
       <c r="F25">
         <v>36.049999999999997</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G25" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1125,7 +1258,7 @@
         <v>2157</v>
       </c>
       <c r="C26" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D26">
         <v>25</v>
@@ -1136,8 +1269,11 @@
       <c r="F26">
         <v>50.56</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G26" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1145,7 +1281,7 @@
         <v>6828</v>
       </c>
       <c r="C27" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1156,8 +1292,11 @@
       <c r="F27">
         <v>36.18</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G27" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1165,7 +1304,7 @@
         <v>1964</v>
       </c>
       <c r="C28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D28">
         <v>25</v>
@@ -1176,8 +1315,11 @@
       <c r="F28">
         <v>54.45</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G28" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1185,7 +1327,7 @@
         <v>6959</v>
       </c>
       <c r="C29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -1196,8 +1338,11 @@
       <c r="F29">
         <v>25.72</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1205,7 +1350,7 @@
         <v>4069</v>
       </c>
       <c r="C30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1216,8 +1361,11 @@
       <c r="F30">
         <v>45.33</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G30" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1225,7 +1373,7 @@
         <v>6897</v>
       </c>
       <c r="C31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D31">
         <v>25</v>
@@ -1236,8 +1384,11 @@
       <c r="F31">
         <v>9.35</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G31" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1245,7 +1396,7 @@
         <v>9233</v>
       </c>
       <c r="C32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -1256,8 +1407,11 @@
       <c r="F32">
         <v>33.78</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G32" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1265,7 +1419,7 @@
         <v>6491</v>
       </c>
       <c r="C33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D33">
         <v>25</v>
@@ -1276,8 +1430,11 @@
       <c r="F33">
         <v>42.31</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G33" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1285,7 +1442,7 @@
         <v>2793</v>
       </c>
       <c r="C34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D34">
         <v>0</v>
@@ -1296,8 +1453,11 @@
       <c r="F34">
         <v>26.45</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G34" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1305,7 +1465,7 @@
         <v>1871</v>
       </c>
       <c r="C35" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D35">
         <v>25</v>
@@ -1316,8 +1476,11 @@
       <c r="F35">
         <v>20</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G35" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1325,7 +1488,7 @@
         <v>5753</v>
       </c>
       <c r="C36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -1336,8 +1499,11 @@
       <c r="F36">
         <v>33.17</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G36" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1345,7 +1511,7 @@
         <v>3677</v>
       </c>
       <c r="C37" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D37">
         <v>25</v>
@@ -1356,8 +1522,11 @@
       <c r="F37">
         <v>28.76</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G37" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1365,7 +1534,7 @@
         <v>6628</v>
       </c>
       <c r="C38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D38">
         <v>0</v>
@@ -1376,8 +1545,11 @@
       <c r="F38">
         <v>31.43</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G38" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1385,7 +1557,7 @@
         <v>4427</v>
       </c>
       <c r="C39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D39">
         <v>25</v>
@@ -1396,8 +1568,11 @@
       <c r="F39">
         <v>43.08</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G39" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1405,7 +1580,7 @@
         <v>6101</v>
       </c>
       <c r="C40" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -1416,8 +1591,11 @@
       <c r="F40">
         <v>25.09</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G40" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1425,7 +1603,7 @@
         <v>499</v>
       </c>
       <c r="C41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D41">
         <v>25</v>
@@ -1436,8 +1614,11 @@
       <c r="F41">
         <v>43.01</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G41" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1445,7 +1626,7 @@
         <v>5885</v>
       </c>
       <c r="C42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -1456,8 +1637,11 @@
       <c r="F42">
         <v>15.21</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G42" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1465,7 +1649,7 @@
         <v>7495</v>
       </c>
       <c r="C43" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D43">
         <v>25</v>
@@ -1476,8 +1660,11 @@
       <c r="F43">
         <v>43.14</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G43" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1485,7 +1672,7 @@
         <v>9689</v>
       </c>
       <c r="C44" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D44">
         <v>0</v>
@@ -1496,8 +1683,11 @@
       <c r="F44">
         <v>22.63</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G44" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1505,7 +1695,7 @@
         <v>5583</v>
       </c>
       <c r="C45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D45">
         <v>25</v>
@@ -1517,7 +1707,7 @@
         <v>30.13</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1525,7 +1715,7 @@
         <v>7492</v>
       </c>
       <c r="C46" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -1537,7 +1727,7 @@
         <v>12.97</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1545,7 +1735,7 @@
         <v>1071</v>
       </c>
       <c r="C47" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D47">
         <v>25</v>
@@ -1556,8 +1746,11 @@
       <c r="F47">
         <v>24.450000000000003</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G47" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1565,7 +1758,7 @@
         <v>899</v>
       </c>
       <c r="C48" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -1576,8 +1769,11 @@
       <c r="F48">
         <v>28.26</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G48" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1585,7 +1781,7 @@
         <v>2595</v>
       </c>
       <c r="C49" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D49">
         <v>25</v>
@@ -1596,8 +1792,11 @@
       <c r="F49">
         <v>22.5</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G49" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1605,7 +1804,7 @@
         <v>2440</v>
       </c>
       <c r="C50" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D50">
         <v>0</v>
@@ -1616,8 +1815,11 @@
       <c r="F50">
         <v>15.74</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G50" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1625,7 +1827,7 @@
         <v>8763</v>
       </c>
       <c r="C51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D51">
         <v>25</v>
@@ -1636,8 +1838,11 @@
       <c r="F51">
         <v>50.45</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G51" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1645,7 +1850,7 @@
         <v>4212</v>
       </c>
       <c r="C52" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D52">
         <v>0</v>
@@ -1656,8 +1861,11 @@
       <c r="F52">
         <v>18.05</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G52" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>53</v>
       </c>
@@ -1665,7 +1873,7 @@
         <v>2065</v>
       </c>
       <c r="C53" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D53">
         <v>25</v>
@@ -1676,8 +1884,11 @@
       <c r="F53">
         <v>50.269999999999996</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G53" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>54</v>
       </c>
@@ -1685,7 +1896,7 @@
         <v>9627</v>
       </c>
       <c r="C54" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D54">
         <v>0</v>
@@ -1696,8 +1907,11 @@
       <c r="F54">
         <v>9.89</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G54" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>55</v>
       </c>
@@ -1705,7 +1919,7 @@
         <v>3113</v>
       </c>
       <c r="C55" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D55">
         <v>25</v>
@@ -1716,8 +1930,11 @@
       <c r="F55">
         <v>59.05</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G55" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>56</v>
       </c>
@@ -1725,7 +1942,7 @@
         <v>7972</v>
       </c>
       <c r="C56" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -1736,8 +1953,11 @@
       <c r="F56">
         <v>14.669999999999998</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G56" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>57</v>
       </c>
@@ -1745,7 +1965,7 @@
         <v>9624</v>
       </c>
       <c r="C57" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D57">
         <v>25</v>
@@ -1756,8 +1976,11 @@
       <c r="F57">
         <v>36.06</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G57" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>58</v>
       </c>
@@ -1765,7 +1988,7 @@
         <v>5694</v>
       </c>
       <c r="C58" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D58">
         <v>0</v>
@@ -1776,8 +1999,11 @@
       <c r="F58">
         <v>31.84</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G58" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>59</v>
       </c>
@@ -1785,7 +2011,7 @@
         <v>4121</v>
       </c>
       <c r="C59" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D59">
         <v>25</v>
@@ -1796,8 +2022,11 @@
       <c r="F59">
         <v>20.86</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G59" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>60</v>
       </c>
@@ -1805,7 +2034,7 @@
         <v>7471</v>
       </c>
       <c r="C60" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -1816,8 +2045,11 @@
       <c r="F60">
         <v>14.73</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G60" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>61</v>
       </c>
@@ -1825,7 +2057,7 @@
         <v>1472</v>
       </c>
       <c r="C61" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D61">
         <v>25</v>
@@ -1836,8 +2068,11 @@
       <c r="F61">
         <v>23.56</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G61" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>62</v>
       </c>
@@ -1845,7 +2080,7 @@
         <v>2172</v>
       </c>
       <c r="C62" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -1856,8 +2091,11 @@
       <c r="F62">
         <v>4.0199999999999996</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G62" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>63</v>
       </c>
@@ -1865,7 +2103,7 @@
         <v>9239</v>
       </c>
       <c r="C63" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D63">
         <v>25</v>
@@ -1876,8 +2114,11 @@
       <c r="F63">
         <v>36.19</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G63" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>64</v>
       </c>
@@ -1885,7 +2126,7 @@
         <v>4558</v>
       </c>
       <c r="C64" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -1896,8 +2137,11 @@
       <c r="F64">
         <v>18.64</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G64" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>65</v>
       </c>
@@ -1905,7 +2149,7 @@
         <v>7064</v>
       </c>
       <c r="C65" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D65">
         <v>25</v>
@@ -1916,8 +2160,11 @@
       <c r="F65">
         <v>24.01</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G65" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>66</v>
       </c>
@@ -1925,7 +2172,7 @@
         <v>3386</v>
       </c>
       <c r="C66" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D66">
         <v>0</v>
@@ -1936,8 +2183,11 @@
       <c r="F66">
         <v>11.62</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G66" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>67</v>
       </c>
@@ -1945,7 +2195,7 @@
         <v>8819</v>
       </c>
       <c r="C67" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D67">
         <v>25</v>
@@ -1956,8 +2206,11 @@
       <c r="F67">
         <v>42.84</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G67" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>68</v>
       </c>
@@ -1965,7 +2218,7 @@
         <v>9591</v>
       </c>
       <c r="C68" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D68">
         <v>0</v>
@@ -1976,41 +2229,44 @@
       <c r="F68">
         <v>33.1</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="G68" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B80" s="1"/>
     </row>
     <row r="81" spans="2:2" ht="16" x14ac:dyDescent="0.2">

</xml_diff>